<commit_message>
feat: v2 — household (spouse SS + healthcare, dependents), per-line real growth, time-boxed expense windows
Additive v1->v2 migration: existing data migrates with zero change to any number
(verified against real data). Spouse contributes their own Social Security and
healthcare on their own age trajectory; dependents drive time-boxed spending.
Growth is real (vs inflation), 0 = grows with inflation = prior behavior.
XLSX template gains a Household tab + growth/window columns; imports round-trip.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -7,7 +7,8 @@
     <sheet name="Properties" sheetId="2" r:id="rId2"/>
     <sheet name="Income" sheetId="3" r:id="rId3"/>
     <sheet name="Spending" sheetId="4" r:id="rId4"/>
-    <sheet name="Assumptions" sheetId="5" r:id="rId5"/>
+    <sheet name="Household" sheetId="5" r:id="rId5"/>
+    <sheet name="Assumptions" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -432,7 +433,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -441,6 +442,8 @@
     <col min="5" max="5" width="13.83203125" customWidth="1"/>
     <col min="6" max="6" width="33.83203125" customWidth="1"/>
     <col min="7" max="7" width="21.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,22 +468,29 @@
       <c r="G1" t="str">
         <v>Net sale proceeds $</v>
       </c>
+      <c r="H1" t="str">
+        <v>Rent real growth %/yr</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Costs real growth %/yr</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="12.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -496,20 +506,26 @@
       <c r="D1" t="str">
         <v>To year</v>
       </c>
+      <c r="E1" t="str">
+        <v>Real growth %/yr</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:E1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
+    <col min="3" max="3" width="32.83203125" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -519,15 +535,75 @@
       <c r="B1" t="str">
         <v>$/mo (excl. property costs &amp; healthcare)</v>
       </c>
+      <c r="C1" t="str">
+        <v>From year (blank = from start)</v>
+      </c>
+      <c r="D1" t="str">
+        <v>To year (blank = perpetual)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Real growth %/yr</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I1"/>
+  <cols>
+    <col min="1" max="1" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="17.83203125" customWidth="1"/>
+    <col min="9" max="9" width="29.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Name</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Role (spouse or dependent)</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Current age</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SS start age</v>
+      </c>
+      <c r="E1" t="str">
+        <v>SS $/mo (pre-haircut)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>SS haircut %</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Health pre-65 $/yr</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Health 65+ $/yr</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Employer coverage until age</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C15"/>
   <cols>

</xml_diff>

<commit_message>
feat: v3 — dependent lump-sum costs, auto-detected current year, collapsible trends, math explainer
- Dependents now carry a one-time lump-sum cost + the year it lands (college,
  a wedding); the do-nothing age field is dropped from the dependent form.
  Ongoing dependent costs still go in Spending. Additive v2->v3 migration
  (verified identical on real data).
- Current year auto-detects at the server boundary via reanchorYears (the
  engine/model stay clock-free); fresh/placeholder state anchors to the real
  year and shifts example years with it. Saved plans are never re-anchored.
- Trends collapses by default (was taking too much space).
- New 'How the math works' section: precise, plain-language description of
  exactly what goes into the calculation.

XLSX Household tab gains lump-sum columns and round-trips. 207 tests pass
including the headless-Chrome render smoke test.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -554,17 +554,19 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="17.83203125" customWidth="1"/>
-    <col min="9" max="9" width="29.83203125" customWidth="1"/>
+    <col min="7" max="7" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="20.83203125" customWidth="1"/>
+    <col min="10" max="10" width="17.83203125" customWidth="1"/>
+    <col min="11" max="11" width="29.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,27 +580,33 @@
         <v>Current age</v>
       </c>
       <c r="D1" t="str">
+        <v>Lump-sum cost $</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Lump-sum year</v>
+      </c>
+      <c r="F1" t="str">
         <v>SS start age</v>
       </c>
-      <c r="E1" t="str">
+      <c r="G1" t="str">
         <v>SS $/mo (pre-haircut)</v>
       </c>
-      <c r="F1" t="str">
+      <c r="H1" t="str">
         <v>SS haircut %</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Health pre-65 $/yr</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>Health 65+ $/yr</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Employer coverage until age</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: dependent support is an ongoing annual cost over a window, not a lump sum
Corrects the v3 dependent model: instead of a one-time lump sum, a dependent
carries an ongoing annual support cost (today's $/yr) over a from/through-year
window — raising a kid for 18 years, supporting a parent until end of life.
The cost behaves like a living expense (flexes with the spending shock, holds
in real terms). Additive v3->v4 migration converts any v3 lump sum losslessly
to a one-year window; verified identical on real data. XLSX Household tab gains
support-cost + from/through columns and round-trips. 207 tests pass incl. the
headless-Chrome smoke test.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -554,19 +554,20 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="19.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.83203125" customWidth="1"/>
     <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="23.83203125" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="17.83203125" customWidth="1"/>
-    <col min="11" max="11" width="29.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="11" max="11" width="17.83203125" customWidth="1"/>
+    <col min="12" max="12" width="29.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -580,33 +581,36 @@
         <v>Current age</v>
       </c>
       <c r="D1" t="str">
-        <v>Lump-sum cost $</v>
+        <v>Support cost $/yr</v>
       </c>
       <c r="E1" t="str">
-        <v>Lump-sum year</v>
+        <v>From year</v>
       </c>
       <c r="F1" t="str">
+        <v>Through year</v>
+      </c>
+      <c r="G1" t="str">
         <v>SS start age</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>SS $/mo (pre-haircut)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>SS haircut %</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Health pre-65 $/yr</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Health 65+ $/yr</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Employer coverage until age</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Own-fund accounts, contribution years, Household profile layout
- Accounts choose "Bucket plan" or "Own fund". An own fund (e.g. a
  target-date 401(k)) earns its own return (default 7% before inflation),
  stays out of the recommended split, and counts as long-term money,
  lowering the bucket plan's equities target. Within a tax type,
  bucket-plan money is withdrawn before own-fund money. The market-crash
  stress drops own funds by the full equity drop.
- Contributions run for "how many more years" instead of until an age.
  The work-until age now only sets the "or earn" window and lives in the
  stress-test card.
- Schema v7 with a v6 -> v7 migration (until-age -> years; a 401(k) moves
  to its own fund).
- Profile, Social Security, healthcare, spouse and dependents are one
  "Household profile" card; Goal moves to the end of the inputs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -402,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:J1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="49.83203125" customWidth="1"/>
@@ -410,8 +410,10 @@
     <col min="4" max="4" width="54.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
     <col min="6" max="6" width="21.83203125" customWidth="1"/>
-    <col min="7" max="7" width="47.83203125" customWidth="1"/>
+    <col min="7" max="7" width="36.83203125" customWidth="1"/>
     <col min="8" max="8" width="48.83203125" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="10" max="10" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,15 +436,21 @@
         <v>Employer match $/yr</v>
       </c>
       <c r="G1" t="str">
-        <v>Contribute until age (blank = work-until age)</v>
+        <v>Contribute for how many more years</v>
       </c>
       <c r="H1" t="str">
         <v>Contribution increase %/yr (blank = inflation)</v>
       </c>
+      <c r="I1" t="str">
+        <v>Invested in (buckets or own)</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Own fund return %/yr (used when invested in own)</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -879,7 +887,7 @@
         <v>50</v>
       </c>
       <c r="C22" t="str">
-        <v>willing-to-work-until age (the solver's income window)</v>
+        <v>for the 'or earn $X/yr' answer: extra income is earned through this age</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
Proportional split, shared plan-to age, remove work-until, reorder inputs
- The split always keeps the bucket targets' proportions: extra money is
  spread the same way instead of all going to equities, so capital
  preservation grows as fewer years remain.
- You and a spouse each live to the plan-to age; the plan runs until the
  younger reaches it. Each person's Social Security and healthcare stop at
  that age, and the survivor keeps the larger Social Security check.
- Removed the work-until age and the "or earn $X/yr" answer (schema v8
  migration; old spreadsheets with the setting still import). Trend rows
  (v3) now track the gap.
- Inputs reordered: Household profile, Income streams, Returns & inflation,
  Portfolio (renamed from Accounts), Taxes, Spending, Properties, Goal.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -641,7 +641,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C22"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -881,23 +881,12 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>work.untilAge</v>
-      </c>
-      <c r="B22">
-        <v>50</v>
-      </c>
-      <c r="C22" t="str">
-        <v>for the 'or earn $X/yr' answer: extra income is earned through this age</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
         <v># Amounts are in today's dollars; rates are actual (before inflation)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Spend more scenario on variable lines; late-life allocation moves gains, not principal
- Spending lines get a 'variable' checkbox. The spend more scenario raises only
  checked lines by a % you set (default 20), as a lasting step-up. Household
  support (childcare), housing, property tax etc. stay put.
- With fewer than the high income cutoff years left, equity gains move to
  capital preservation instead of rebalancing; in the final capital preservation
  years, high income gains move too. Principal is only tapped to top up capital
  preservation after an up year.
- Schema v10 migration guesses variable flags from line names.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -495,13 +495,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
     <col min="3" max="3" width="32.83203125" customWidth="1"/>
     <col min="4" max="4" width="29.83203125" customWidth="1"/>
     <col min="5" max="5" width="35.83203125" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,10 +521,13 @@
       <c r="E1" t="str">
         <v>Increase %/yr (blank = inflation)</v>
       </c>
+      <c r="F1" t="str">
+        <v>Variable (yes/no)</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -593,7 +597,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -660,7 +664,7 @@
         <v>buckets.preservationReturnPct</v>
       </c>
       <c r="B6">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C6" t="str">
         <v>capital preservation return %/yr, before inflation</v>
@@ -671,7 +675,7 @@
         <v>buckets.incomeReturnPct</v>
       </c>
       <c r="B7">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="C7" t="str">
         <v>high income return %/yr, before inflation</v>
@@ -682,7 +686,7 @@
         <v>buckets.equitiesReturnPct</v>
       </c>
       <c r="B8">
-        <v>9.5</v>
+        <v>8</v>
       </c>
       <c r="C8" t="str">
         <v>global equities return %/yr, before inflation</v>
@@ -756,133 +760,144 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>taxes.ordinaryIncomePct</v>
+        <v>simulation.spendMorePct</v>
       </c>
       <c r="B15">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C15" t="str">
-        <v>effective tax % on traditional IRA / 401(k) withdrawals (federal + state)</v>
+        <v>spend more scenario: % increase on variable spending lines</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>taxes.capitalGainsPct</v>
+        <v>taxes.ordinaryIncomePct</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C16" t="str">
-        <v>effective tax % on gains when selling in a taxable account (federal + state)</v>
+        <v>effective tax % on traditional IRA / 401(k) withdrawals (federal + state)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>social.startAge</v>
+        <v>taxes.capitalGainsPct</v>
       </c>
       <c r="B17">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="C17" t="str">
-        <v>Social Security start age (years)</v>
+        <v>effective tax % on gains when selling in a taxable account (federal + state)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>social.monthly</v>
+        <v>social.startAge</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="C18" t="str">
-        <v>Social Security $/mo, today's dollars, pre-haircut</v>
+        <v>Social Security start age (years)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>social.haircutPct</v>
+        <v>social.monthly</v>
       </c>
       <c r="B19">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C19" t="str">
-        <v>% cut applied to Social Security (plain number, 25 = 25%)</v>
+        <v>Social Security $/mo, today's dollars, pre-haircut</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>health.preMedicareAnnual</v>
+        <v>social.haircutPct</v>
       </c>
       <c r="B20">
-        <v>16000</v>
+        <v>25</v>
       </c>
       <c r="C20" t="str">
-        <v>healthcare $/yr before 65, after employer coverage ends</v>
+        <v>% cut applied to Social Security (plain number, 25 = 25%)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>health.postMedicareAnnual</v>
+        <v>health.preMedicareAnnual</v>
       </c>
       <c r="B21">
-        <v>7500</v>
+        <v>16000</v>
       </c>
       <c r="C21" t="str">
-        <v>healthcare $/yr from age 65</v>
+        <v>healthcare $/yr before 65, after employer coverage ends</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>health.employerCoverageUntilAge</v>
+        <v>health.postMedicareAnnual</v>
       </c>
       <c r="B22">
-        <v>40</v>
+        <v>7500</v>
       </c>
       <c r="C22" t="str">
-        <v>age employer health coverage ends</v>
+        <v>healthcare $/yr from age 65</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>endState.mode</v>
-      </c>
-      <c r="B23" t="str">
-        <v>zero</v>
+        <v>health.employerCoverageUntilAge</v>
+      </c>
+      <c r="B23">
+        <v>40</v>
       </c>
       <c r="C23" t="str">
-        <v>one of: zero, bequest, floor</v>
+        <v>age employer health coverage ends</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>endState.bequest</v>
-      </c>
-      <c r="B24">
-        <v>0</v>
+        <v>endState.mode</v>
+      </c>
+      <c r="B24" t="str">
+        <v>zero</v>
       </c>
       <c r="C24" t="str">
-        <v>$ to leave (used when mode is bequest)</v>
+        <v>one of: zero, bequest, floor</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>endState.floor</v>
+        <v>endState.bequest</v>
       </c>
       <c r="B25">
         <v>0</v>
       </c>
       <c r="C25" t="str">
-        <v>$ the balance never drops below (used when mode is floor)</v>
+        <v>$ to leave (used when mode is bequest)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>endState.floor</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26" t="str">
+        <v>$ the balance never drops below (used when mode is floor)</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
         <v># Amounts are in today's dollars; rates are actual (before inflation)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dedicated-bucket accounts replace own funds
- An account is invested in the bucket plan or dedicated to one bucket
  (capital preservation, high income, global equities). A dedicated account
  earns that bucket's return and swing (moving with it in every simulated
  year) and counts toward that bucket's target; the bucket plan fills the rest
  and is the only money rebalanced.
- Results show the total asset allocation and, when accounts are dedicated,
  the bucket plan allocation (how to invest the rest).
- Within a tax type, spending comes from dedicated capital preservation, the
  bucket plan, dedicated high income, then dedicated equities.
- Schema v12: own-fund accounts move to the bucket with the closest swing.
- Smoke test waits for the simulated futures instead of a fixed 4s.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:J1"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="49.83203125" customWidth="1"/>
@@ -411,10 +411,8 @@
     <col min="6" max="6" width="21.83203125" customWidth="1"/>
     <col min="7" max="7" width="36.83203125" customWidth="1"/>
     <col min="8" max="8" width="48.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
-    <col min="11" max="11" width="49.83203125" customWidth="1"/>
-    <col min="12" max="12" width="34.83203125" customWidth="1"/>
+    <col min="9" max="9" width="58.83203125" customWidth="1"/>
+    <col min="10" max="10" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -443,21 +441,15 @@
         <v>Contribution increase %/yr (blank = inflation)</v>
       </c>
       <c r="I1" t="str">
-        <v>Invested in (buckets or own)</v>
+        <v>Invested in (buckets, preservation, income, or equities)</v>
       </c>
       <c r="J1" t="str">
-        <v>Own fund return %/yr (used when invested in own)</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Own fund swing %/yr (used when invested in own)</v>
-      </c>
-      <c r="L1" t="str">
         <v>Owner (self or spouse; for RMDs)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Retirement money only counts toward years from its owner's 59½; IRAs default to high income
- Money in a traditional IRA, 401(k) or Roth (dedicated or not) only counts
  toward the part of a bucket's target for years its owner is 59½ or older.
  The part for earlier years must be covered by taxable money, so the bucket
  plan holds it, and the results say how much of the bucket plan to keep in
  taxable accounts (and whether there's enough).
- Topping up the safe buckets from a dedicated retirement account likewise
  only covers years from the owner's 59½.
- The 10% early-withdrawal penalty follows the account owner's age.
- Roth accounts get an owner too.
- Traditional IRAs default to high income; schema v13 moves traditional IRAs
  in the bucket plan to high income.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -412,7 +412,7 @@
     <col min="7" max="7" width="36.83203125" customWidth="1"/>
     <col min="8" max="8" width="48.83203125" customWidth="1"/>
     <col min="9" max="9" width="58.83203125" customWidth="1"/>
-    <col min="10" max="10" width="34.83203125" customWidth="1"/>
+    <col min="10" max="10" width="42.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -444,7 +444,7 @@
         <v>Invested in (buckets, preservation, income, or equities)</v>
       </c>
       <c r="J1" t="str">
-        <v>Owner (self or spouse; for RMDs)</v>
+        <v>Owner (self or spouse; for RMDs and 59½)</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show capital preservation in three layers: cash, short-term bonds, medium-term
Two new cutoffs (cash through year 1, short-term bonds through year 4 by
default); medium-term runs to the capital preservation cutoff. The results
show each layer's dollars under capital preservation, for the total asset
allocation and the bucket plan allocation, soonest years filled first.
Display only: capital preservation keeps one return and swing. Schema v14.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -593,7 +593,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -701,199 +701,221 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>buckets.incomeThroughYear</v>
+        <v>buckets.cashYears</v>
       </c>
       <c r="B10">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="C10" t="str">
-        <v>high income holds years N+1 through this year; equities hold the rest</v>
+        <v>within capital preservation: years 1 to C as cash (shown in the results only)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>buckets.preservationVolPct</v>
+        <v>buckets.shortBondYears</v>
       </c>
       <c r="B11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11" t="str">
-        <v>capital preservation's typical yearly swing %, for the simulation</v>
+        <v>within capital preservation: years C+1 to S in short-term bonds; the rest medium-term (shown in the results only)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>buckets.incomeVolPct</v>
+        <v>buckets.incomeThroughYear</v>
       </c>
       <c r="B12">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="C12" t="str">
-        <v>high income's typical yearly swing %</v>
+        <v>high income holds years N+1 through this year; equities hold the rest</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>buckets.equitiesVolPct</v>
+        <v>buckets.preservationVolPct</v>
       </c>
       <c r="B13">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="C13" t="str">
-        <v>global equities' typical yearly swing %</v>
+        <v>capital preservation's typical yearly swing %, for the simulation</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>simulation.targetSuccessPct</v>
+        <v>buckets.incomeVolPct</v>
       </c>
       <c r="B14">
-        <v>90</v>
+        <v>8</v>
       </c>
       <c r="C14" t="str">
-        <v>the plan should work in this % of simulated futures (the gap aims for it)</v>
+        <v>high income's typical yearly swing %</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>simulation.spendMorePct</v>
+        <v>buckets.equitiesVolPct</v>
       </c>
       <c r="B15">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C15" t="str">
-        <v>spend more scenario: % increase on variable spending lines</v>
+        <v>global equities' typical yearly swing %</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>taxes.ordinaryIncomePct</v>
+        <v>simulation.targetSuccessPct</v>
       </c>
       <c r="B16">
-        <v>22</v>
+        <v>90</v>
       </c>
       <c r="C16" t="str">
-        <v>effective tax % on traditional IRA / 401(k) withdrawals (federal + state)</v>
+        <v>the plan should work in this % of simulated futures (the gap aims for it)</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>taxes.capitalGainsPct</v>
+        <v>simulation.spendMorePct</v>
       </c>
       <c r="B17">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C17" t="str">
-        <v>effective tax % on gains when selling in a taxable account (federal + state)</v>
+        <v>spend more scenario: % increase on variable spending lines</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>social.startAge</v>
+        <v>taxes.ordinaryIncomePct</v>
       </c>
       <c r="B18">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="C18" t="str">
-        <v>Social Security start age (years)</v>
+        <v>effective tax % on traditional IRA / 401(k) withdrawals (federal + state)</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>social.monthly</v>
+        <v>taxes.capitalGainsPct</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="C19" t="str">
-        <v>Social Security $/mo, today's dollars, pre-haircut</v>
+        <v>effective tax % on gains when selling in a taxable account (federal + state)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>social.haircutPct</v>
+        <v>social.startAge</v>
       </c>
       <c r="B20">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="C20" t="str">
-        <v>% cut applied to Social Security (plain number, 25 = 25%)</v>
+        <v>Social Security start age (years)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>health.preMedicareAnnual</v>
+        <v>social.monthly</v>
       </c>
       <c r="B21">
-        <v>16000</v>
+        <v>0</v>
       </c>
       <c r="C21" t="str">
-        <v>healthcare $/yr before 65, after employer coverage ends</v>
+        <v>Social Security $/mo, today's dollars, pre-haircut</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>health.postMedicareAnnual</v>
+        <v>social.haircutPct</v>
       </c>
       <c r="B22">
-        <v>7500</v>
+        <v>25</v>
       </c>
       <c r="C22" t="str">
-        <v>healthcare $/yr from age 65</v>
+        <v>% cut applied to Social Security (plain number, 25 = 25%)</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>health.employerCoverageUntilAge</v>
+        <v>health.preMedicareAnnual</v>
       </c>
       <c r="B23">
-        <v>40</v>
+        <v>16000</v>
       </c>
       <c r="C23" t="str">
-        <v>age employer health coverage ends</v>
+        <v>healthcare $/yr before 65, after employer coverage ends</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>endState.mode</v>
-      </c>
-      <c r="B24" t="str">
-        <v>zero</v>
+        <v>health.postMedicareAnnual</v>
+      </c>
+      <c r="B24">
+        <v>7500</v>
       </c>
       <c r="C24" t="str">
-        <v>one of: zero, bequest, floor</v>
+        <v>healthcare $/yr from age 65</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>endState.bequest</v>
+        <v>health.employerCoverageUntilAge</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C25" t="str">
-        <v>$ to leave (used when mode is bequest)</v>
+        <v>age employer health coverage ends</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>endState.floor</v>
-      </c>
-      <c r="B26">
-        <v>0</v>
+        <v>endState.mode</v>
+      </c>
+      <c r="B26" t="str">
+        <v>zero</v>
       </c>
       <c r="C26" t="str">
-        <v>$ the balance never drops below (used when mode is floor)</v>
+        <v>one of: zero, bequest, floor</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>endState.bequest</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="C27" t="str">
+        <v>$ to leave (used when mode is bequest)</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>endState.floor</v>
+      </c>
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="C28" t="str">
+        <v>$ the balance never drops below (used when mode is floor)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
         <v># Amounts are in today's dollars; rates are actual (before inflation)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Liquid years: a rolling window replaces the strict 59½ rule
While an account's owner is under 59½, retirement-account money doesn't
count toward the next N years of withdrawals (default 10); it counts toward
every later year, and toward every year from 59½ on. So an IRA in high
income counts toward the later high income years while the brokerage keeps
the near-term years liquid. The results also say how far taxable money alone
reaches ("covers withdrawals through age X"). Schema v15.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01X8EHkkgm5uZdJ9v5F1FsKn
</commit_message>
<xml_diff>
--- a/template/runway-template.xlsx
+++ b/template/runway-template.xlsx
@@ -593,7 +593,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -712,210 +712,221 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>buckets.shortBondYears</v>
+        <v>buckets.liquidYears</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C11" t="str">
-        <v>within capital preservation: years C+1 to S in short-term bonds; the rest medium-term (shown in the results only)</v>
+        <v>while under 59½, the next N years of withdrawals must be covered by taxable accounts</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>buckets.incomeThroughYear</v>
+        <v>buckets.shortBondYears</v>
       </c>
       <c r="B12">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="C12" t="str">
-        <v>high income holds years N+1 through this year; equities hold the rest</v>
+        <v>within capital preservation: years C+1 to S in short-term bonds; the rest medium-term (shown in the results only)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>buckets.preservationVolPct</v>
+        <v>buckets.incomeThroughYear</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C13" t="str">
-        <v>capital preservation's typical yearly swing %, for the simulation</v>
+        <v>high income holds years N+1 through this year; equities hold the rest</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>buckets.incomeVolPct</v>
+        <v>buckets.preservationVolPct</v>
       </c>
       <c r="B14">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C14" t="str">
-        <v>high income's typical yearly swing %</v>
+        <v>capital preservation's typical yearly swing %, for the simulation</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>buckets.equitiesVolPct</v>
+        <v>buckets.incomeVolPct</v>
       </c>
       <c r="B15">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C15" t="str">
-        <v>global equities' typical yearly swing %</v>
+        <v>high income's typical yearly swing %</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>simulation.targetSuccessPct</v>
+        <v>buckets.equitiesVolPct</v>
       </c>
       <c r="B16">
-        <v>90</v>
+        <v>17</v>
       </c>
       <c r="C16" t="str">
-        <v>the plan should work in this % of simulated futures (the gap aims for it)</v>
+        <v>global equities' typical yearly swing %</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>simulation.spendMorePct</v>
+        <v>simulation.targetSuccessPct</v>
       </c>
       <c r="B17">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="C17" t="str">
-        <v>spend more scenario: % increase on variable spending lines</v>
+        <v>the plan should work in this % of simulated futures (the gap aims for it)</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>taxes.ordinaryIncomePct</v>
+        <v>simulation.spendMorePct</v>
       </c>
       <c r="B18">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C18" t="str">
-        <v>effective tax % on traditional IRA / 401(k) withdrawals (federal + state)</v>
+        <v>spend more scenario: % increase on variable spending lines</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>taxes.capitalGainsPct</v>
+        <v>taxes.ordinaryIncomePct</v>
       </c>
       <c r="B19">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C19" t="str">
-        <v>effective tax % on gains when selling in a taxable account (federal + state)</v>
+        <v>effective tax % on traditional IRA / 401(k) withdrawals (federal + state)</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>social.startAge</v>
+        <v>taxes.capitalGainsPct</v>
       </c>
       <c r="B20">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="C20" t="str">
-        <v>Social Security start age (years)</v>
+        <v>effective tax % on gains when selling in a taxable account (federal + state)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>social.monthly</v>
+        <v>social.startAge</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="C21" t="str">
-        <v>Social Security $/mo, today's dollars, pre-haircut</v>
+        <v>Social Security start age (years)</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>social.haircutPct</v>
+        <v>social.monthly</v>
       </c>
       <c r="B22">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="C22" t="str">
-        <v>% cut applied to Social Security (plain number, 25 = 25%)</v>
+        <v>Social Security $/mo, today's dollars, pre-haircut</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>health.preMedicareAnnual</v>
+        <v>social.haircutPct</v>
       </c>
       <c r="B23">
-        <v>16000</v>
+        <v>25</v>
       </c>
       <c r="C23" t="str">
-        <v>healthcare $/yr before 65, after employer coverage ends</v>
+        <v>% cut applied to Social Security (plain number, 25 = 25%)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>health.postMedicareAnnual</v>
+        <v>health.preMedicareAnnual</v>
       </c>
       <c r="B24">
-        <v>7500</v>
+        <v>16000</v>
       </c>
       <c r="C24" t="str">
-        <v>healthcare $/yr from age 65</v>
+        <v>healthcare $/yr before 65, after employer coverage ends</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>health.employerCoverageUntilAge</v>
+        <v>health.postMedicareAnnual</v>
       </c>
       <c r="B25">
-        <v>40</v>
+        <v>7500</v>
       </c>
       <c r="C25" t="str">
-        <v>age employer health coverage ends</v>
+        <v>healthcare $/yr from age 65</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>endState.mode</v>
-      </c>
-      <c r="B26" t="str">
-        <v>zero</v>
+        <v>health.employerCoverageUntilAge</v>
+      </c>
+      <c r="B26">
+        <v>40</v>
       </c>
       <c r="C26" t="str">
-        <v>one of: zero, bequest, floor</v>
+        <v>age employer health coverage ends</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>endState.bequest</v>
-      </c>
-      <c r="B27">
-        <v>0</v>
+        <v>endState.mode</v>
+      </c>
+      <c r="B27" t="str">
+        <v>zero</v>
       </c>
       <c r="C27" t="str">
-        <v>$ to leave (used when mode is bequest)</v>
+        <v>one of: zero, bequest, floor</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>endState.floor</v>
+        <v>endState.bequest</v>
       </c>
       <c r="B28">
         <v>0</v>
       </c>
       <c r="C28" t="str">
-        <v>$ the balance never drops below (used when mode is floor)</v>
+        <v>$ to leave (used when mode is bequest)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
+        <v>endState.floor</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="C29" t="str">
+        <v>$ the balance never drops below (used when mode is floor)</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
         <v># Amounts are in today's dollars; rates are actual (before inflation)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>